<commit_message>
Final set v1.6: product-specific output elasticities (cement -0.10); documents on mirror numbers, kernel v1.6 and rebuild v0.5 builders drafted
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MnaF19gSWzaMiztLqS74jT
</commit_message>
<xml_diff>
--- a/egypt-final/simple/Egypt_Simple.xlsx
+++ b/egypt-final/simple/Egypt_Simple.xlsx
@@ -135,7 +135,7 @@
     <xf numFmtId="1" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -815,22 +815,22 @@
         </is>
       </c>
       <c r="B9" s="10" t="n">
-        <v>-7.2908</v>
+        <v>-4.5615</v>
       </c>
       <c r="C9" s="10" t="n">
-        <v>-2.9782</v>
+        <v>-1.8279</v>
       </c>
       <c r="D9" s="10" t="n">
-        <v>-3.05</v>
+        <v>-1.9008</v>
       </c>
       <c r="E9" s="10" t="n">
-        <v>-7.2908</v>
+        <v>-4.5615</v>
       </c>
       <c r="F9" s="10" t="n">
         <v>-3.6649</v>
       </c>
       <c r="G9" s="10" t="n">
-        <v>-17.5641</v>
+        <v>-15.3548</v>
       </c>
     </row>
     <row r="10">
@@ -911,22 +911,22 @@
         </is>
       </c>
       <c r="B15" s="10" t="n">
-        <v>6.8595</v>
+        <v>6.914</v>
       </c>
       <c r="C15" s="10" t="n">
-        <v>6.2669</v>
+        <v>6.2756</v>
       </c>
       <c r="D15" s="10" t="n">
-        <v>6.2294</v>
+        <v>6.2382</v>
       </c>
       <c r="E15" s="10" t="n">
-        <v>1.5352</v>
+        <v>1.5898</v>
       </c>
       <c r="F15" s="10" t="n">
         <v>0.3157</v>
       </c>
       <c r="G15" s="10" t="n">
-        <v>0.4061</v>
+        <v>0.4057</v>
       </c>
     </row>
     <row r="16">
@@ -936,22 +936,22 @@
         </is>
       </c>
       <c r="B16" s="13" t="n">
-        <v>1501.1341</v>
+        <v>1440.3299</v>
       </c>
       <c r="C16" s="13" t="n">
-        <v>1456.3479</v>
+        <v>1430.8363</v>
       </c>
       <c r="D16" s="13" t="n">
-        <v>1517.1987</v>
+        <v>1492.0462</v>
       </c>
       <c r="E16" s="13" t="n">
-        <v>551.5895</v>
+        <v>508.523</v>
       </c>
       <c r="F16" s="13" t="n">
         <v>329.7507</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>646.3092</v>
+        <v>606.5145</v>
       </c>
     </row>
     <row r="17">
@@ -1192,11 +1192,11 @@
         </is>
       </c>
       <c r="B8" s="21" t="n">
-        <v>-0.5</v>
+        <v>-0.1</v>
       </c>
       <c r="C8" s="19" t="inlineStr">
         <is>
-          <t>-0.5 means 1% dearer gives 0.5% less output. A rough placeholder.</t>
+          <t>-0.1 for cement: 1% dearer gives 0.1% less output. Steel and fertiliser -0.4, aluminium -0.5. Based on studies of demand and pass-through.</t>
         </is>
       </c>
     </row>

</xml_diff>